<commit_message>
feat(app): add short video adaptive launcher icon and use i18n app_name
- Add modern short video adaptive launcher icons (ic_launcher_background, ic_launcher_foreground, mipmap-anydpi-v26)
- Configure android:icon and android:roundIcon in AndroidManifest.xml
- Update app and activity label to @string/app_name
- Update i18n/strings.xlsx and regenerate localized strings.xml (English: 'Short Video', Chinese: '短视频')
</commit_message>
<xml_diff>
--- a/i18n/strings.xlsx
+++ b/i18n/strings.xlsx
@@ -446,12 +446,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>My App</t>
+          <t>Short Video</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>我的应用</t>
+          <t>短视频</t>
         </is>
       </c>
     </row>

</xml_diff>